<commit_message>
Fix Excel UID scientific notation and hidden dates in downloads.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/xlsx/monthly.xlsx
+++ b/docs/xlsx/monthly.xlsx
@@ -15,6 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -73,9 +76,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -374,6 +380,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -394,7 +401,7 @@
           <t>2021-07</t>
         </is>
       </c>
-      <c r="B2">
+      <c r="B2" s="2">
         <v>108045</v>
       </c>
     </row>
@@ -404,7 +411,7 @@
           <t>2021-08</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" s="2">
         <v>347263</v>
       </c>
     </row>
@@ -414,7 +421,7 @@
           <t>2021-09</t>
         </is>
       </c>
-      <c r="B4">
+      <c r="B4" s="2">
         <v>1631</v>
       </c>
     </row>
@@ -424,7 +431,7 @@
           <t>2021-10</t>
         </is>
       </c>
-      <c r="B5">
+      <c r="B5" s="2">
         <v>1270</v>
       </c>
     </row>
@@ -434,7 +441,7 @@
           <t>2021-11</t>
         </is>
       </c>
-      <c r="B6">
+      <c r="B6" s="2">
         <v>460</v>
       </c>
     </row>
@@ -444,7 +451,7 @@
           <t>2021-12</t>
         </is>
       </c>
-      <c r="B7">
+      <c r="B7" s="2">
         <v>557</v>
       </c>
     </row>
@@ -454,7 +461,7 @@
           <t>2022-01</t>
         </is>
       </c>
-      <c r="B8">
+      <c r="B8" s="2">
         <v>1594</v>
       </c>
     </row>
@@ -464,7 +471,7 @@
           <t>2022-02</t>
         </is>
       </c>
-      <c r="B9">
+      <c r="B9" s="2">
         <v>1217</v>
       </c>
     </row>
@@ -474,7 +481,7 @@
           <t>2022-03</t>
         </is>
       </c>
-      <c r="B10">
+      <c r="B10" s="2">
         <v>895</v>
       </c>
     </row>
@@ -484,7 +491,7 @@
           <t>2022-04</t>
         </is>
       </c>
-      <c r="B11">
+      <c r="B11" s="2">
         <v>1075</v>
       </c>
     </row>
@@ -494,7 +501,7 @@
           <t>2022-05</t>
         </is>
       </c>
-      <c r="B12">
+      <c r="B12" s="2">
         <v>832</v>
       </c>
     </row>
@@ -504,7 +511,7 @@
           <t>2022-06</t>
         </is>
       </c>
-      <c r="B13">
+      <c r="B13" s="2">
         <v>1553</v>
       </c>
     </row>
@@ -514,7 +521,7 @@
           <t>2022-07</t>
         </is>
       </c>
-      <c r="B14">
+      <c r="B14" s="2">
         <v>5278</v>
       </c>
     </row>
@@ -524,7 +531,7 @@
           <t>2022-08</t>
         </is>
       </c>
-      <c r="B15">
+      <c r="B15" s="2">
         <v>1334</v>
       </c>
     </row>
@@ -534,7 +541,7 @@
           <t>2022-09</t>
         </is>
       </c>
-      <c r="B16">
+      <c r="B16" s="2">
         <v>174</v>
       </c>
     </row>
@@ -544,7 +551,7 @@
           <t>2022-10</t>
         </is>
       </c>
-      <c r="B17">
+      <c r="B17" s="2">
         <v>233</v>
       </c>
     </row>
@@ -554,7 +561,7 @@
           <t>2022-11</t>
         </is>
       </c>
-      <c r="B18">
+      <c r="B18" s="2">
         <v>211</v>
       </c>
     </row>
@@ -564,7 +571,7 @@
           <t>2022-12</t>
         </is>
       </c>
-      <c r="B19">
+      <c r="B19" s="2">
         <v>477</v>
       </c>
     </row>
@@ -574,7 +581,7 @@
           <t>2023-01</t>
         </is>
       </c>
-      <c r="B20">
+      <c r="B20" s="2">
         <v>681</v>
       </c>
     </row>
@@ -584,7 +591,7 @@
           <t>2023-02</t>
         </is>
       </c>
-      <c r="B21">
+      <c r="B21" s="2">
         <v>373</v>
       </c>
     </row>
@@ -594,7 +601,7 @@
           <t>2023-03</t>
         </is>
       </c>
-      <c r="B22">
+      <c r="B22" s="2">
         <v>219</v>
       </c>
     </row>
@@ -604,7 +611,7 @@
           <t>2023-04</t>
         </is>
       </c>
-      <c r="B23">
+      <c r="B23" s="2">
         <v>384</v>
       </c>
     </row>
@@ -614,7 +621,7 @@
           <t>2023-05</t>
         </is>
       </c>
-      <c r="B24">
+      <c r="B24" s="2">
         <v>336</v>
       </c>
     </row>
@@ -624,7 +631,7 @@
           <t>2023-06</t>
         </is>
       </c>
-      <c r="B25">
+      <c r="B25" s="2">
         <v>367</v>
       </c>
     </row>
@@ -634,7 +641,7 @@
           <t>2023-07</t>
         </is>
       </c>
-      <c r="B26">
+      <c r="B26" s="2">
         <v>751</v>
       </c>
     </row>
@@ -644,7 +651,7 @@
           <t>2023-08</t>
         </is>
       </c>
-      <c r="B27">
+      <c r="B27" s="2">
         <v>366</v>
       </c>
     </row>
@@ -654,7 +661,7 @@
           <t>2023-09</t>
         </is>
       </c>
-      <c r="B28">
+      <c r="B28" s="2">
         <v>448</v>
       </c>
     </row>
@@ -664,7 +671,7 @@
           <t>2023-10</t>
         </is>
       </c>
-      <c r="B29">
+      <c r="B29" s="2">
         <v>381</v>
       </c>
     </row>
@@ -674,7 +681,7 @@
           <t>2023-11</t>
         </is>
       </c>
-      <c r="B30">
+      <c r="B30" s="2">
         <v>752</v>
       </c>
     </row>
@@ -684,7 +691,7 @@
           <t>2023-12</t>
         </is>
       </c>
-      <c r="B31">
+      <c r="B31" s="2">
         <v>139</v>
       </c>
     </row>
@@ -694,7 +701,7 @@
           <t>2024-01</t>
         </is>
       </c>
-      <c r="B32">
+      <c r="B32" s="2">
         <v>236</v>
       </c>
     </row>
@@ -704,7 +711,7 @@
           <t>2024-02</t>
         </is>
       </c>
-      <c r="B33">
+      <c r="B33" s="2">
         <v>409</v>
       </c>
     </row>
@@ -714,7 +721,7 @@
           <t>2024-03</t>
         </is>
       </c>
-      <c r="B34">
+      <c r="B34" s="2">
         <v>263</v>
       </c>
     </row>
@@ -724,7 +731,7 @@
           <t>2024-04</t>
         </is>
       </c>
-      <c r="B35">
+      <c r="B35" s="2">
         <v>580</v>
       </c>
     </row>
@@ -734,7 +741,7 @@
           <t>2024-05</t>
         </is>
       </c>
-      <c r="B36">
+      <c r="B36" s="2">
         <v>375</v>
       </c>
     </row>
@@ -744,7 +751,7 @@
           <t>2024-06</t>
         </is>
       </c>
-      <c r="B37">
+      <c r="B37" s="2">
         <v>562</v>
       </c>
     </row>
@@ -754,7 +761,7 @@
           <t>2024-07</t>
         </is>
       </c>
-      <c r="B38">
+      <c r="B38" s="2">
         <v>3437</v>
       </c>
     </row>
@@ -764,7 +771,7 @@
           <t>2024-08</t>
         </is>
       </c>
-      <c r="B39">
+      <c r="B39" s="2">
         <v>3196</v>
       </c>
     </row>
@@ -774,7 +781,7 @@
           <t>2024-09</t>
         </is>
       </c>
-      <c r="B40">
+      <c r="B40" s="2">
         <v>160</v>
       </c>
     </row>
@@ -784,7 +791,7 @@
           <t>2024-10</t>
         </is>
       </c>
-      <c r="B41">
+      <c r="B41" s="2">
         <v>155</v>
       </c>
     </row>
@@ -794,7 +801,7 @@
           <t>2024-11</t>
         </is>
       </c>
-      <c r="B42">
+      <c r="B42" s="2">
         <v>207</v>
       </c>
     </row>
@@ -804,7 +811,7 @@
           <t>2024-12</t>
         </is>
       </c>
-      <c r="B43">
+      <c r="B43" s="2">
         <v>202</v>
       </c>
     </row>
@@ -814,7 +821,7 @@
           <t>2025-01</t>
         </is>
       </c>
-      <c r="B44">
+      <c r="B44" s="2">
         <v>236</v>
       </c>
     </row>
@@ -824,7 +831,7 @@
           <t>2025-02</t>
         </is>
       </c>
-      <c r="B45">
+      <c r="B45" s="2">
         <v>264</v>
       </c>
     </row>
@@ -834,7 +841,7 @@
           <t>2025-03</t>
         </is>
       </c>
-      <c r="B46">
+      <c r="B46" s="2">
         <v>445</v>
       </c>
     </row>
@@ -844,7 +851,7 @@
           <t>2025-04</t>
         </is>
       </c>
-      <c r="B47">
+      <c r="B47" s="2">
         <v>24996</v>
       </c>
     </row>
@@ -854,7 +861,7 @@
           <t>2025-05</t>
         </is>
       </c>
-      <c r="B48">
+      <c r="B48" s="2">
         <v>4669</v>
       </c>
     </row>
@@ -864,7 +871,7 @@
           <t>2025-06</t>
         </is>
       </c>
-      <c r="B49">
+      <c r="B49" s="2">
         <v>22039</v>
       </c>
     </row>
@@ -874,7 +881,7 @@
           <t>2025-07</t>
         </is>
       </c>
-      <c r="B50">
+      <c r="B50" s="2">
         <v>13596</v>
       </c>
     </row>
@@ -884,7 +891,7 @@
           <t>2025-08</t>
         </is>
       </c>
-      <c r="B51">
+      <c r="B51" s="2">
         <v>3991</v>
       </c>
     </row>
@@ -894,7 +901,7 @@
           <t>2025-09</t>
         </is>
       </c>
-      <c r="B52">
+      <c r="B52" s="2">
         <v>1166</v>
       </c>
     </row>
@@ -904,7 +911,7 @@
           <t>2025-10</t>
         </is>
       </c>
-      <c r="B53">
+      <c r="B53" s="2">
         <v>183684</v>
       </c>
     </row>
@@ -914,7 +921,7 @@
           <t>2025-11</t>
         </is>
       </c>
-      <c r="B54">
+      <c r="B54" s="2">
         <v>22569</v>
       </c>
     </row>
@@ -924,7 +931,7 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="B55">
+      <c r="B55" s="2">
         <v>8927</v>
       </c>
     </row>
@@ -934,7 +941,7 @@
           <t>2026-01</t>
         </is>
       </c>
-      <c r="B56">
+      <c r="B56" s="2">
         <v>9336</v>
       </c>
     </row>
@@ -944,7 +951,7 @@
           <t>2026-02</t>
         </is>
       </c>
-      <c r="B57">
+      <c r="B57" s="2">
         <v>3410608</v>
       </c>
     </row>
@@ -954,7 +961,7 @@
           <t>2026-03</t>
         </is>
       </c>
-      <c r="B58">
+      <c r="B58" s="2">
         <v>142694</v>
       </c>
     </row>
@@ -964,7 +971,7 @@
           <t>2026-04</t>
         </is>
       </c>
-      <c r="B59">
+      <c r="B59" s="2">
         <v>256819</v>
       </c>
     </row>
@@ -974,7 +981,7 @@
           <t>2026-05</t>
         </is>
       </c>
-      <c r="B60">
+      <c r="B60" s="2">
         <v>130764</v>
       </c>
     </row>
@@ -984,7 +991,7 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="B61">
+      <c r="B61" s="2">
         <v>68448</v>
       </c>
     </row>
@@ -994,7 +1001,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="B62">
+      <c r="B62" s="2">
         <v>179479</v>
       </c>
     </row>
@@ -1004,7 +1011,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="B63">
+      <c r="B63" s="2">
         <v>62884</v>
       </c>
     </row>

</xml_diff>